<commit_message>
HW: Schematics rearranged for documentation, half-bridge control signals moved to layer Mid 4, additional netclass added for terminals (protection against the spread of fire), terminal position fixed (2mm offset in height), clearance adjusted for 600V CAT II
</commit_message>
<xml_diff>
--- a/hw/Terminal_offset.xlsx
+++ b/hw/Terminal_offset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Daten\Daniel\ele\bat_source\hw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B84D832-0AEF-4B1C-A945-629A4F0B6E8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE074F38-E60B-4434-B641-9D8BE7414BD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17325" xr2:uid="{7FE45C81-C561-428F-9A74-EE5EFF6E3519}"/>
   </bookViews>
@@ -78,12 +78,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -98,8 +104,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1230,21 +1237,21 @@
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>19</v>
-      </c>
-      <c r="B22">
+      <c r="A22" s="1">
+        <v>19</v>
+      </c>
+      <c r="B22" s="1">
         <v>2</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="1">
         <f t="shared" si="0"/>
         <v>18.894443627691185</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="1">
         <f t="shared" si="1"/>
         <v>18.899999999999999</v>
       </c>
-      <c r="E22">
+      <c r="E22" s="1">
         <f t="shared" si="2"/>
         <v>5.5563723088134509E-3</v>
       </c>
@@ -11532,8 +11539,8 @@
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
-        <cfvo type="percentile" val="5"/>
         <cfvo type="percentile" val="10"/>
+        <cfvo type="percentile" val="20"/>
         <color rgb="FF63BE7B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FFF8696B"/>

</xml_diff>